<commit_message>
Cập nhật bảng chia tiền điện miễn phí (bắt lỗi nhập chính xác hơn)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9SwcTtPPFTYwK8QkVLdBg
</commit_message>
<xml_diff>
--- a/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
+++ b/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t xml:space="preserve">CHIA TIỀN ĐIỆN NHÀ TRỌ THEO HÓA ĐƠN – BẢN MIỄN PHÍ</t>
   </si>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Xong thì sang tab 'Giấy báo': mỗi phòng một đoạn ghi rõ cách tính, chép gửi Zalo cho người thuê.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sang tháng mới: Tạo bản sao file (hoặc bản sao tab 'Tính tiền'), chép cột 'Điện mới' sang cột 'cũ', xóa số tháng trước.</t>
+    <t xml:space="preserve">Sang tháng mới: Tạo bản sao file (hoặc bản sao tab 'Tính tiền'), chép cột 'Điện mới' sang cột 'Điện cũ', xóa số tháng trước.</t>
   </si>
   <si>
     <t xml:space="preserve">Hai cách chia điện (đều không vượt hóa đơn):</t>
@@ -79,7 +79,10 @@
     <t xml:space="preserve">Bản đầy đủ có thêm:</t>
   </si>
   <si>
-    <t xml:space="preserve">• Tiền nước (theo đồng hồ hoặc theo người), tiền phòng, phí dịch vụ, nợ tháng trước, đã thu / còn nợ.</t>
+    <t xml:space="preserve">• Sổ cả năm 12 tháng: chỉ số cũ và nợ tự chuyển sang tháng sau, tab tổng kết cả năm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tiền nước (theo đồng hồ hoặc theo người), tiền phòng, phí dịch vụ, nợ, đã thu / còn nợ; nhắc hợp đồng sắp hết hạn.</t>
   </si>
   <si>
     <t xml:space="preserve">• Giấy báo tổng tiền từng phòng gồm tất cả các khoản.</t>
@@ -128,6 +131,9 @@
   </si>
   <si>
     <t xml:space="preserve">Tiền điện</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giấy báo (tự tạo)</t>
   </si>
   <si>
     <t xml:space="preserve">P101</t>
@@ -309,84 +315,88 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -658,128 +668,136 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="130"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3"/>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
+      <c r="A7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
+      <c r="A14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
+      <c r="A16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-    </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="A24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -798,115 +816,119 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>20</v>
+      <c r="A1" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>22</v>
       </c>
+      <c r="B3" s="6" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="8" t="n">
+      <c r="A4" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="7" t="n">
         <v>1980000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="8" t="n">
         <v>700</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="10" t="n">
+      <c r="A6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="9" t="n">
         <f aca="false">IF(B5&gt;0,B4/B5,0)</f>
         <v>2828.57142857143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="11" t="n">
+      <c r="A7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="10" t="n">
         <f aca="false">SUM(E12:E41)</f>
         <v>655</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="12" t="n">
+      <c r="A8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="11" t="n">
         <f aca="false">SUM(F12:F41)</f>
         <v>1852600</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="13" t="str">
-        <f aca="false">IF(B4&lt;=0,"Nhập số tiền và kWh trên hóa đơn điện lực",IF(SUMPRODUCT(--ISTEXT(C12:D41))&gt;0,"LỖI: có ô chỉ số điện không phải số (gõ chữ hoặc dấu chấm) – chỉ gõ số",IF(SUMPRODUCT((C12:C41&lt;&gt;"")*(D12:D41&lt;&gt;"")*(D12:D41&lt;C12:C41))&gt;0,"LỖI: có phòng chỉ số điện mới nhỏ hơn chỉ số cũ – kiểm tra lại",IF(B8&gt;B4,"VƯỢT HÓA ĐƠN: đang thu "&amp;TEXT(B8-B4,"#,##0")&amp;" đ nhiều hơn hóa đơn – không được thu",IF(AND(NOT('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng"),B7&gt;B5),"VƯỢT: tổng kWh các phòng lớn hơn kWh trên hóa đơn – kiểm tra chỉ số hoặc công tơ","ĐÚNG: tổng tiền điện thu "&amp;TEXT(B8,"#,##0")&amp;" đ ≤ hóa đơn "&amp;TEXT(B4,"#,##0")&amp;" đ")))))</f>
+      <c r="A9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="12" t="str">
+        <f aca="false">IF(B4&lt;=0,"Nhập số tiền và kWh trên hóa đơn điện lực",IF(SUMPRODUCT(ISTEXT(C12:D41)*(C12:D41&lt;&gt;""))&gt;0,"LỖI: có ô chỉ số điện không phải số (gõ chữ hoặc dấu chấm) – chỉ gõ số",IF(SUMPRODUCT((C12:C41&lt;&gt;"")*(D12:D41&lt;&gt;"")*(D12:D41&lt;C12:C41))&gt;0,"LỖI: có phòng chỉ số điện mới nhỏ hơn chỉ số cũ – kiểm tra lại",IF(B8&gt;B4,"VƯỢT HÓA ĐƠN: đang thu "&amp;TEXT(B8-B4,"#,##0")&amp;" đ nhiều hơn hóa đơn – không được thu",IF(AND(NOT('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng"),B7&gt;B5),"VƯỢT: tổng kWh các phòng lớn hơn kWh trên hóa đơn – kiểm tra chỉ số hoặc công tơ","ĐÚNG: tổng tiền điện thu "&amp;TEXT(B8,"#,##0")&amp;" đ ≤ hóa đơn "&amp;TEXT(B4,"#,##0")&amp;" đ")))))</f>
         <v>ĐÚNG: tổng tiền điện thu 1,852,600 đ ≤ hóa đơn 1,980,000 đ</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="A11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="B11" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="C11" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="E11" s="13" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F11" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>1200</v>
@@ -922,13 +944,19 @@
         <f aca="false">IF(E12=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E12/$B$7,-2),0),ROUNDDOWN(E12*$B$6,-2)))</f>
         <v>622200</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G12" s="19" t="str">
+        <f aca="false">IF(OR(A12="",$B$4&lt;=0),"","Phòng "&amp;A12&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C12,"#,##0")&amp;" → "&amp;TEXT(D12,"#,##0")&amp;" = "&amp;E12&amp;" kWh → "&amp;TEXT(F12,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E12&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v>Phòng P101 – tháng 10/2026
+Điện: 1,200 → 1,420 = 220 kWh → 622,200 đ
+(Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>850</v>
@@ -944,13 +972,19 @@
         <f aca="false">IF(E13=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E13/$B$7,-2),0),ROUNDDOWN(E13*$B$6,-2)))</f>
         <v>396000</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G13" s="19" t="str">
+        <f aca="false">IF(OR(A13="",$B$4&lt;=0),"","Phòng "&amp;A13&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C13,"#,##0")&amp;" → "&amp;TEXT(D13,"#,##0")&amp;" = "&amp;E13&amp;" kWh → "&amp;TEXT(F13,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E13&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v>Phòng P102 – tháng 10/2026
+Điện: 850 → 990 = 140 kWh → 396,000 đ
+(Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>3010</v>
@@ -966,8 +1000,14 @@
         <f aca="false">IF(E14=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E14/$B$7,-2),0),ROUNDDOWN(E14*$B$6,-2)))</f>
         <v>834400</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G14" s="19" t="str">
+        <f aca="false">IF(OR(A14="",$B$4&lt;=0),"","Phòng "&amp;A14&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C14,"#,##0")&amp;" → "&amp;TEXT(D14,"#,##0")&amp;" = "&amp;E14&amp;" kWh → "&amp;TEXT(F14,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E14&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v>Phòng P103 – tháng 10/2026
+Điện: 3,010 → 3,305 = 295 kWh → 834,400 đ
+(Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="16"/>
@@ -980,8 +1020,12 @@
         <f aca="false">IF(E15=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E15/$B$7,-2),0),ROUNDDOWN(E15*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G15" s="19" t="str">
+        <f aca="false">IF(OR(A15="",$B$4&lt;=0),"","Phòng "&amp;A15&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C15,"#,##0")&amp;" → "&amp;TEXT(D15,"#,##0")&amp;" = "&amp;E15&amp;" kWh → "&amp;TEXT(F15,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E15&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="16"/>
@@ -994,8 +1038,12 @@
         <f aca="false">IF(E16=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E16/$B$7,-2),0),ROUNDDOWN(E16*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G16" s="19" t="str">
+        <f aca="false">IF(OR(A16="",$B$4&lt;=0),"","Phòng "&amp;A16&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C16,"#,##0")&amp;" → "&amp;TEXT(D16,"#,##0")&amp;" = "&amp;E16&amp;" kWh → "&amp;TEXT(F16,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E16&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="16"/>
@@ -1008,8 +1056,12 @@
         <f aca="false">IF(E17=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E17/$B$7,-2),0),ROUNDDOWN(E17*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G17" s="19" t="str">
+        <f aca="false">IF(OR(A17="",$B$4&lt;=0),"","Phòng "&amp;A17&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C17,"#,##0")&amp;" → "&amp;TEXT(D17,"#,##0")&amp;" = "&amp;E17&amp;" kWh → "&amp;TEXT(F17,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E17&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="16"/>
@@ -1022,8 +1074,12 @@
         <f aca="false">IF(E18=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E18/$B$7,-2),0),ROUNDDOWN(E18*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G18" s="19" t="str">
+        <f aca="false">IF(OR(A18="",$B$4&lt;=0),"","Phòng "&amp;A18&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C18,"#,##0")&amp;" → "&amp;TEXT(D18,"#,##0")&amp;" = "&amp;E18&amp;" kWh → "&amp;TEXT(F18,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E18&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="16"/>
@@ -1036,8 +1092,12 @@
         <f aca="false">IF(E19=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E19/$B$7,-2),0),ROUNDDOWN(E19*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G19" s="19" t="str">
+        <f aca="false">IF(OR(A19="",$B$4&lt;=0),"","Phòng "&amp;A19&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C19,"#,##0")&amp;" → "&amp;TEXT(D19,"#,##0")&amp;" = "&amp;E19&amp;" kWh → "&amp;TEXT(F19,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E19&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15"/>
       <c r="B20" s="15"/>
       <c r="C20" s="16"/>
@@ -1050,8 +1110,12 @@
         <f aca="false">IF(E20=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E20/$B$7,-2),0),ROUNDDOWN(E20*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G20" s="19" t="str">
+        <f aca="false">IF(OR(A20="",$B$4&lt;=0),"","Phòng "&amp;A20&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C20,"#,##0")&amp;" → "&amp;TEXT(D20,"#,##0")&amp;" = "&amp;E20&amp;" kWh → "&amp;TEXT(F20,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E20&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15"/>
       <c r="B21" s="15"/>
       <c r="C21" s="16"/>
@@ -1064,8 +1128,12 @@
         <f aca="false">IF(E21=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E21/$B$7,-2),0),ROUNDDOWN(E21*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G21" s="19" t="str">
+        <f aca="false">IF(OR(A21="",$B$4&lt;=0),"","Phòng "&amp;A21&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C21,"#,##0")&amp;" → "&amp;TEXT(D21,"#,##0")&amp;" = "&amp;E21&amp;" kWh → "&amp;TEXT(F21,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E21&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15"/>
       <c r="B22" s="15"/>
       <c r="C22" s="16"/>
@@ -1078,8 +1146,12 @@
         <f aca="false">IF(E22=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E22/$B$7,-2),0),ROUNDDOWN(E22*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G22" s="19" t="str">
+        <f aca="false">IF(OR(A22="",$B$4&lt;=0),"","Phòng "&amp;A22&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C22,"#,##0")&amp;" → "&amp;TEXT(D22,"#,##0")&amp;" = "&amp;E22&amp;" kWh → "&amp;TEXT(F22,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E22&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15"/>
       <c r="B23" s="15"/>
       <c r="C23" s="16"/>
@@ -1092,8 +1164,12 @@
         <f aca="false">IF(E23=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E23/$B$7,-2),0),ROUNDDOWN(E23*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G23" s="19" t="str">
+        <f aca="false">IF(OR(A23="",$B$4&lt;=0),"","Phòng "&amp;A23&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C23,"#,##0")&amp;" → "&amp;TEXT(D23,"#,##0")&amp;" = "&amp;E23&amp;" kWh → "&amp;TEXT(F23,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E23&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15"/>
       <c r="B24" s="15"/>
       <c r="C24" s="16"/>
@@ -1106,8 +1182,12 @@
         <f aca="false">IF(E24=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E24/$B$7,-2),0),ROUNDDOWN(E24*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G24" s="19" t="str">
+        <f aca="false">IF(OR(A24="",$B$4&lt;=0),"","Phòng "&amp;A24&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C24,"#,##0")&amp;" → "&amp;TEXT(D24,"#,##0")&amp;" = "&amp;E24&amp;" kWh → "&amp;TEXT(F24,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E24&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15"/>
       <c r="B25" s="15"/>
       <c r="C25" s="16"/>
@@ -1120,8 +1200,12 @@
         <f aca="false">IF(E25=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E25/$B$7,-2),0),ROUNDDOWN(E25*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G25" s="19" t="str">
+        <f aca="false">IF(OR(A25="",$B$4&lt;=0),"","Phòng "&amp;A25&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C25,"#,##0")&amp;" → "&amp;TEXT(D25,"#,##0")&amp;" = "&amp;E25&amp;" kWh → "&amp;TEXT(F25,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E25&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15"/>
       <c r="B26" s="15"/>
       <c r="C26" s="16"/>
@@ -1134,8 +1218,12 @@
         <f aca="false">IF(E26=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E26/$B$7,-2),0),ROUNDDOWN(E26*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G26" s="19" t="str">
+        <f aca="false">IF(OR(A26="",$B$4&lt;=0),"","Phòng "&amp;A26&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C26,"#,##0")&amp;" → "&amp;TEXT(D26,"#,##0")&amp;" = "&amp;E26&amp;" kWh → "&amp;TEXT(F26,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E26&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15"/>
       <c r="B27" s="15"/>
       <c r="C27" s="16"/>
@@ -1148,8 +1236,12 @@
         <f aca="false">IF(E27=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E27/$B$7,-2),0),ROUNDDOWN(E27*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G27" s="19" t="str">
+        <f aca="false">IF(OR(A27="",$B$4&lt;=0),"","Phòng "&amp;A27&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C27,"#,##0")&amp;" → "&amp;TEXT(D27,"#,##0")&amp;" = "&amp;E27&amp;" kWh → "&amp;TEXT(F27,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E27&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="15"/>
       <c r="B28" s="15"/>
       <c r="C28" s="16"/>
@@ -1162,8 +1254,12 @@
         <f aca="false">IF(E28=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E28/$B$7,-2),0),ROUNDDOWN(E28*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G28" s="19" t="str">
+        <f aca="false">IF(OR(A28="",$B$4&lt;=0),"","Phòng "&amp;A28&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C28,"#,##0")&amp;" → "&amp;TEXT(D28,"#,##0")&amp;" = "&amp;E28&amp;" kWh → "&amp;TEXT(F28,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E28&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="15"/>
       <c r="B29" s="15"/>
       <c r="C29" s="16"/>
@@ -1176,8 +1272,12 @@
         <f aca="false">IF(E29=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E29/$B$7,-2),0),ROUNDDOWN(E29*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G29" s="19" t="str">
+        <f aca="false">IF(OR(A29="",$B$4&lt;=0),"","Phòng "&amp;A29&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C29,"#,##0")&amp;" → "&amp;TEXT(D29,"#,##0")&amp;" = "&amp;E29&amp;" kWh → "&amp;TEXT(F29,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E29&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="15"/>
       <c r="B30" s="15"/>
       <c r="C30" s="16"/>
@@ -1190,8 +1290,12 @@
         <f aca="false">IF(E30=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E30/$B$7,-2),0),ROUNDDOWN(E30*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G30" s="19" t="str">
+        <f aca="false">IF(OR(A30="",$B$4&lt;=0),"","Phòng "&amp;A30&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C30,"#,##0")&amp;" → "&amp;TEXT(D30,"#,##0")&amp;" = "&amp;E30&amp;" kWh → "&amp;TEXT(F30,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E30&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="15"/>
       <c r="B31" s="15"/>
       <c r="C31" s="16"/>
@@ -1204,8 +1308,12 @@
         <f aca="false">IF(E31=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E31/$B$7,-2),0),ROUNDDOWN(E31*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G31" s="19" t="str">
+        <f aca="false">IF(OR(A31="",$B$4&lt;=0),"","Phòng "&amp;A31&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C31,"#,##0")&amp;" → "&amp;TEXT(D31,"#,##0")&amp;" = "&amp;E31&amp;" kWh → "&amp;TEXT(F31,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E31&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="15"/>
       <c r="B32" s="15"/>
       <c r="C32" s="16"/>
@@ -1218,8 +1326,12 @@
         <f aca="false">IF(E32=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E32/$B$7,-2),0),ROUNDDOWN(E32*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G32" s="19" t="str">
+        <f aca="false">IF(OR(A32="",$B$4&lt;=0),"","Phòng "&amp;A32&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C32,"#,##0")&amp;" → "&amp;TEXT(D32,"#,##0")&amp;" = "&amp;E32&amp;" kWh → "&amp;TEXT(F32,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E32&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="15"/>
       <c r="B33" s="15"/>
       <c r="C33" s="16"/>
@@ -1232,8 +1344,12 @@
         <f aca="false">IF(E33=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E33/$B$7,-2),0),ROUNDDOWN(E33*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G33" s="19" t="str">
+        <f aca="false">IF(OR(A33="",$B$4&lt;=0),"","Phòng "&amp;A33&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C33,"#,##0")&amp;" → "&amp;TEXT(D33,"#,##0")&amp;" = "&amp;E33&amp;" kWh → "&amp;TEXT(F33,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E33&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="15"/>
       <c r="B34" s="15"/>
       <c r="C34" s="16"/>
@@ -1246,8 +1362,12 @@
         <f aca="false">IF(E34=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E34/$B$7,-2),0),ROUNDDOWN(E34*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G34" s="19" t="str">
+        <f aca="false">IF(OR(A34="",$B$4&lt;=0),"","Phòng "&amp;A34&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C34,"#,##0")&amp;" → "&amp;TEXT(D34,"#,##0")&amp;" = "&amp;E34&amp;" kWh → "&amp;TEXT(F34,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E34&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="15"/>
       <c r="B35" s="15"/>
       <c r="C35" s="16"/>
@@ -1260,8 +1380,12 @@
         <f aca="false">IF(E35=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E35/$B$7,-2),0),ROUNDDOWN(E35*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G35" s="19" t="str">
+        <f aca="false">IF(OR(A35="",$B$4&lt;=0),"","Phòng "&amp;A35&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C35,"#,##0")&amp;" → "&amp;TEXT(D35,"#,##0")&amp;" = "&amp;E35&amp;" kWh → "&amp;TEXT(F35,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E35&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="15"/>
       <c r="B36" s="15"/>
       <c r="C36" s="16"/>
@@ -1274,8 +1398,12 @@
         <f aca="false">IF(E36=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E36/$B$7,-2),0),ROUNDDOWN(E36*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G36" s="19" t="str">
+        <f aca="false">IF(OR(A36="",$B$4&lt;=0),"","Phòng "&amp;A36&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C36,"#,##0")&amp;" → "&amp;TEXT(D36,"#,##0")&amp;" = "&amp;E36&amp;" kWh → "&amp;TEXT(F36,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E36&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="15"/>
       <c r="B37" s="15"/>
       <c r="C37" s="16"/>
@@ -1288,8 +1416,12 @@
         <f aca="false">IF(E37=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E37/$B$7,-2),0),ROUNDDOWN(E37*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G37" s="19" t="str">
+        <f aca="false">IF(OR(A37="",$B$4&lt;=0),"","Phòng "&amp;A37&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C37,"#,##0")&amp;" → "&amp;TEXT(D37,"#,##0")&amp;" = "&amp;E37&amp;" kWh → "&amp;TEXT(F37,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E37&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="15"/>
       <c r="B38" s="15"/>
       <c r="C38" s="16"/>
@@ -1302,8 +1434,12 @@
         <f aca="false">IF(E38=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E38/$B$7,-2),0),ROUNDDOWN(E38*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G38" s="19" t="str">
+        <f aca="false">IF(OR(A38="",$B$4&lt;=0),"","Phòng "&amp;A38&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C38,"#,##0")&amp;" → "&amp;TEXT(D38,"#,##0")&amp;" = "&amp;E38&amp;" kWh → "&amp;TEXT(F38,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E38&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="15"/>
       <c r="B39" s="15"/>
       <c r="C39" s="16"/>
@@ -1316,8 +1452,12 @@
         <f aca="false">IF(E39=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E39/$B$7,-2),0),ROUNDDOWN(E39*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G39" s="19" t="str">
+        <f aca="false">IF(OR(A39="",$B$4&lt;=0),"","Phòng "&amp;A39&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C39,"#,##0")&amp;" → "&amp;TEXT(D39,"#,##0")&amp;" = "&amp;E39&amp;" kWh → "&amp;TEXT(F39,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E39&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="15"/>
       <c r="B40" s="15"/>
       <c r="C40" s="16"/>
@@ -1330,8 +1470,12 @@
         <f aca="false">IF(E40=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E40/$B$7,-2),0),ROUNDDOWN(E40*$B$6,-2)))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G40" s="19" t="str">
+        <f aca="false">IF(OR(A40="",$B$4&lt;=0),"","Phòng "&amp;A40&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C40,"#,##0")&amp;" → "&amp;TEXT(D40,"#,##0")&amp;" = "&amp;E40&amp;" kWh → "&amp;TEXT(F40,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E40&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="15"/>
       <c r="B41" s="15"/>
       <c r="C41" s="16"/>
@@ -1344,6 +1488,10 @@
         <f aca="false">IF(E41=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E41/$B$7,-2),0),ROUNDDOWN(E41*$B$6,-2)))</f>
         <v>0</v>
       </c>
+      <c r="G41" s="19" t="str">
+        <f aca="false">IF(OR(A41="",$B$4&lt;=0),"","Phòng "&amp;A41&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C41,"#,##0")&amp;" → "&amp;TEXT(D41,"#,##0")&amp;" = "&amp;E41&amp;" kWh → "&amp;TEXT(F41,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E41&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B9">
@@ -1351,7 +1499,7 @@
       <formula>LEFT(B9,4)="ĐÚNG"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>LEFT(B9,4)&lt;&gt;"ĐÚNG"</formula>
+      <formula>AND(LEFT(B9,4)&lt;&gt;"ĐÚNG",LEFT(B9,4)&lt;&gt;"Nhập")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12:D41">
@@ -1383,202 +1531,202 @@
   <dimension ref="A1:A32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="95"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>41</v>
+      <c r="A1" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>42</v>
+      <c r="A2" s="4" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A12="","","Phòng "&amp;'Tính tiền'!A12&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C12,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D12,"#,##0")&amp;" = "&amp;'Tính tiền'!E12&amp;" kWh → "&amp;TEXT('Tính tiền'!F12,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E12&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A3" s="20" t="str">
+        <f aca="false">'Tính tiền'!G12</f>
         <v>Phòng P101 – tháng 10/2026
 Điện: 1,200 → 1,420 = 220 kWh → 622,200 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A13="","","Phòng "&amp;'Tính tiền'!A13&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C13,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D13,"#,##0")&amp;" = "&amp;'Tính tiền'!E13&amp;" kWh → "&amp;TEXT('Tính tiền'!F13,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E13&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A4" s="20" t="str">
+        <f aca="false">'Tính tiền'!G13</f>
         <v>Phòng P102 – tháng 10/2026
 Điện: 850 → 990 = 140 kWh → 396,000 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A14="","","Phòng "&amp;'Tính tiền'!A14&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C14,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D14,"#,##0")&amp;" = "&amp;'Tính tiền'!E14&amp;" kWh → "&amp;TEXT('Tính tiền'!F14,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E14&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A5" s="20" t="str">
+        <f aca="false">'Tính tiền'!G14</f>
         <v>Phòng P103 – tháng 10/2026
 Điện: 3,010 → 3,305 = 295 kWh → 834,400 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A15="","","Phòng "&amp;'Tính tiền'!A15&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C15,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D15,"#,##0")&amp;" = "&amp;'Tính tiền'!E15&amp;" kWh → "&amp;TEXT('Tính tiền'!F15,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E15&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A6" s="20" t="str">
+        <f aca="false">'Tính tiền'!G15</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A16="","","Phòng "&amp;'Tính tiền'!A16&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C16,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D16,"#,##0")&amp;" = "&amp;'Tính tiền'!E16&amp;" kWh → "&amp;TEXT('Tính tiền'!F16,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E16&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A7" s="20" t="str">
+        <f aca="false">'Tính tiền'!G16</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A17="","","Phòng "&amp;'Tính tiền'!A17&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C17,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D17,"#,##0")&amp;" = "&amp;'Tính tiền'!E17&amp;" kWh → "&amp;TEXT('Tính tiền'!F17,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E17&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A8" s="20" t="str">
+        <f aca="false">'Tính tiền'!G17</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A18="","","Phòng "&amp;'Tính tiền'!A18&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C18,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D18,"#,##0")&amp;" = "&amp;'Tính tiền'!E18&amp;" kWh → "&amp;TEXT('Tính tiền'!F18,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E18&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A9" s="20" t="str">
+        <f aca="false">'Tính tiền'!G18</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A19="","","Phòng "&amp;'Tính tiền'!A19&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C19,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D19,"#,##0")&amp;" = "&amp;'Tính tiền'!E19&amp;" kWh → "&amp;TEXT('Tính tiền'!F19,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E19&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A10" s="20" t="str">
+        <f aca="false">'Tính tiền'!G19</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A20="","","Phòng "&amp;'Tính tiền'!A20&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C20,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D20,"#,##0")&amp;" = "&amp;'Tính tiền'!E20&amp;" kWh → "&amp;TEXT('Tính tiền'!F20,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E20&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A11" s="20" t="str">
+        <f aca="false">'Tính tiền'!G20</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A21="","","Phòng "&amp;'Tính tiền'!A21&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C21,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D21,"#,##0")&amp;" = "&amp;'Tính tiền'!E21&amp;" kWh → "&amp;TEXT('Tính tiền'!F21,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E21&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A12" s="20" t="str">
+        <f aca="false">'Tính tiền'!G21</f>
         <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A22="","","Phòng "&amp;'Tính tiền'!A22&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C22,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D22,"#,##0")&amp;" = "&amp;'Tính tiền'!E22&amp;" kWh → "&amp;TEXT('Tính tiền'!F22,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E22&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A13" s="20" t="str">
+        <f aca="false">'Tính tiền'!G22</f>
         <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A23="","","Phòng "&amp;'Tính tiền'!A23&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C23,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D23,"#,##0")&amp;" = "&amp;'Tính tiền'!E23&amp;" kWh → "&amp;TEXT('Tính tiền'!F23,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E23&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A14" s="20" t="str">
+        <f aca="false">'Tính tiền'!G23</f>
         <v/>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A24="","","Phòng "&amp;'Tính tiền'!A24&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C24,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D24,"#,##0")&amp;" = "&amp;'Tính tiền'!E24&amp;" kWh → "&amp;TEXT('Tính tiền'!F24,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E24&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A15" s="20" t="str">
+        <f aca="false">'Tính tiền'!G24</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A25="","","Phòng "&amp;'Tính tiền'!A25&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C25,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D25,"#,##0")&amp;" = "&amp;'Tính tiền'!E25&amp;" kWh → "&amp;TEXT('Tính tiền'!F25,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E25&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A16" s="20" t="str">
+        <f aca="false">'Tính tiền'!G25</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A26="","","Phòng "&amp;'Tính tiền'!A26&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C26,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D26,"#,##0")&amp;" = "&amp;'Tính tiền'!E26&amp;" kWh → "&amp;TEXT('Tính tiền'!F26,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E26&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A17" s="20" t="str">
+        <f aca="false">'Tính tiền'!G26</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A27="","","Phòng "&amp;'Tính tiền'!A27&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C27,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D27,"#,##0")&amp;" = "&amp;'Tính tiền'!E27&amp;" kWh → "&amp;TEXT('Tính tiền'!F27,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E27&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A18" s="20" t="str">
+        <f aca="false">'Tính tiền'!G27</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A28="","","Phòng "&amp;'Tính tiền'!A28&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C28,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D28,"#,##0")&amp;" = "&amp;'Tính tiền'!E28&amp;" kWh → "&amp;TEXT('Tính tiền'!F28,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E28&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A19" s="20" t="str">
+        <f aca="false">'Tính tiền'!G28</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A29="","","Phòng "&amp;'Tính tiền'!A29&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C29,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D29,"#,##0")&amp;" = "&amp;'Tính tiền'!E29&amp;" kWh → "&amp;TEXT('Tính tiền'!F29,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E29&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A20" s="20" t="str">
+        <f aca="false">'Tính tiền'!G29</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A30="","","Phòng "&amp;'Tính tiền'!A30&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C30,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D30,"#,##0")&amp;" = "&amp;'Tính tiền'!E30&amp;" kWh → "&amp;TEXT('Tính tiền'!F30,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E30&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A21" s="20" t="str">
+        <f aca="false">'Tính tiền'!G30</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A31="","","Phòng "&amp;'Tính tiền'!A31&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C31,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D31,"#,##0")&amp;" = "&amp;'Tính tiền'!E31&amp;" kWh → "&amp;TEXT('Tính tiền'!F31,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E31&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A22" s="20" t="str">
+        <f aca="false">'Tính tiền'!G31</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A32="","","Phòng "&amp;'Tính tiền'!A32&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C32,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D32,"#,##0")&amp;" = "&amp;'Tính tiền'!E32&amp;" kWh → "&amp;TEXT('Tính tiền'!F32,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E32&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A23" s="20" t="str">
+        <f aca="false">'Tính tiền'!G32</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A33="","","Phòng "&amp;'Tính tiền'!A33&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C33,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D33,"#,##0")&amp;" = "&amp;'Tính tiền'!E33&amp;" kWh → "&amp;TEXT('Tính tiền'!F33,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E33&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A24" s="20" t="str">
+        <f aca="false">'Tính tiền'!G33</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A34="","","Phòng "&amp;'Tính tiền'!A34&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C34,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D34,"#,##0")&amp;" = "&amp;'Tính tiền'!E34&amp;" kWh → "&amp;TEXT('Tính tiền'!F34,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E34&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A25" s="20" t="str">
+        <f aca="false">'Tính tiền'!G34</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A35="","","Phòng "&amp;'Tính tiền'!A35&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C35,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D35,"#,##0")&amp;" = "&amp;'Tính tiền'!E35&amp;" kWh → "&amp;TEXT('Tính tiền'!F35,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E35&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A26" s="20" t="str">
+        <f aca="false">'Tính tiền'!G35</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A36="","","Phòng "&amp;'Tính tiền'!A36&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C36,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D36,"#,##0")&amp;" = "&amp;'Tính tiền'!E36&amp;" kWh → "&amp;TEXT('Tính tiền'!F36,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E36&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A27" s="20" t="str">
+        <f aca="false">'Tính tiền'!G36</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A37="","","Phòng "&amp;'Tính tiền'!A37&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C37,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D37,"#,##0")&amp;" = "&amp;'Tính tiền'!E37&amp;" kWh → "&amp;TEXT('Tính tiền'!F37,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E37&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A28" s="20" t="str">
+        <f aca="false">'Tính tiền'!G37</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A38="","","Phòng "&amp;'Tính tiền'!A38&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C38,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D38,"#,##0")&amp;" = "&amp;'Tính tiền'!E38&amp;" kWh → "&amp;TEXT('Tính tiền'!F38,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E38&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A29" s="20" t="str">
+        <f aca="false">'Tính tiền'!G38</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A39="","","Phòng "&amp;'Tính tiền'!A39&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C39,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D39,"#,##0")&amp;" = "&amp;'Tính tiền'!E39&amp;" kWh → "&amp;TEXT('Tính tiền'!F39,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E39&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A30" s="20" t="str">
+        <f aca="false">'Tính tiền'!G39</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A40="","","Phòng "&amp;'Tính tiền'!A40&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C40,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D40,"#,##0")&amp;" = "&amp;'Tính tiền'!E40&amp;" kWh → "&amp;TEXT('Tính tiền'!F40,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E40&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A31" s="20" t="str">
+        <f aca="false">'Tính tiền'!G40</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="19" t="str">
-        <f aca="false">IF('Tính tiền'!A41="","","Phòng "&amp;'Tính tiền'!A41&amp;" – tháng "&amp;'Tính tiền'!$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT('Tính tiền'!C41,"#,##0")&amp;" → "&amp;TEXT('Tính tiền'!D41,"#,##0")&amp;" = "&amp;'Tính tiền'!E41&amp;" kWh → "&amp;TEXT('Tính tiền'!F41,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;'Tính tiền'!E41&amp;" / tổng các phòng "&amp;TEXT('Tính tiền'!$B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT('Tính tiền'!$B$4,"#,##0")&amp;" đ / "&amp;TEXT('Tính tiền'!$B$5,"#,##0")&amp;" kWh = "&amp;TEXT('Tính tiền'!$B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+      <c r="A32" s="20" t="str">
+        <f aca="false">'Tính tiền'!G41</f>
         <v/>
       </c>
     </row>
@@ -1601,29 +1749,29 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>43</v>
+      <c r="A1" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>44</v>
+      <c r="A3" s="12" t="s">
+        <v>46</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>46</v>
+      <c r="A4" s="12" t="s">
+        <v>48</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sửa bài tiền điện phòng trọ: bỏ khẳng định quá mức về mốc hiệu lực Thông tư 60/2025 (theo rà soát pháp chế)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9SwcTtPPFTYwK8QkVLdBg
</commit_message>
<xml_diff>
--- a/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
+++ b/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
@@ -31,13 +31,13 @@
     <t xml:space="preserve">Vì sao cần:</t>
   </si>
   <si>
-    <t xml:space="preserve">Người thuê không ký hợp đồng điện trực tiếp với điện lực thì TỔNG tiền điện chủ nhà thu KHÔNG được vượt số tiền trên hóa đơn điện tháng đó</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(điểm c khoản 5 Điều 12 Thông tư 60/2025/TT-BCT, hiệu lực 02/12/2025). Thu vượt có thể bị phạt 20–30 triệu đồng và buộc hoàn trả (Nghị định 133/2026/NĐ-CP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bảng này chia đúng hóa đơn điện lực cho từng phòng, làm tròn XUỐNG 100 đ, nên tổng thu luôn ≤ hóa đơn.</t>
+    <t xml:space="preserve">Thu tiền điện của người thuê cao hơn giá quy định có thể bị phạt 20–30 triệu đồng và buộc hoàn trả (Nghị định 133/2026/NĐ-CP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông tư 60/2025/TT-BCT (điểm c khoản 5 Điều 12) quy định tổng tiền điện chủ nhà thu không vượt hóa đơn tháng; mốc áp dụng điểm này các nguồn chưa thống nhất – hỏi điện lực nơi bạn ở.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bảng này chia hóa đơn điện lực cho từng phòng, làm tròn XUỐNG 100 đ. Nhập chỉ số đúng thì tổng thu không vượt hóa đơn; ô KIỂM TRA báo đỏ khi vượt.</t>
   </si>
   <si>
     <t xml:space="preserve">Mỗi tháng làm 3 bước (ô nền vàng là ô bạn nhập):</t>

</xml_diff>

<commit_message>
Cập nhật bảng chia tiền điện miễn phí (sửa lỗi do QA độc lập tìm ra)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q9SwcTtPPFTYwK8QkVLdBg
</commit_message>
<xml_diff>
--- a/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
+++ b/tai-ve/chia-tien-dien-nha-tro-mien-phi.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t xml:space="preserve">CHIA TIỀN ĐIỆN NHÀ TRỌ THEO HÓA ĐƠN – BẢN MIỄN PHÍ</t>
   </si>
@@ -55,6 +55,9 @@
     <t xml:space="preserve">   Công tơ quay vòng về 0: ghi Điện cũ = 0 và Điện mới = số kWh phòng đã dùng tháng đó.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Bảng đã khóa cấu trúc (không chèn, xóa, sắp xếp dòng) để công thức không vỡ; mọi ô nền vàng vẫn sửa được. Phòng trống: xóa tên người thuê.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Xong thì sang tab 'Giấy báo': mỗi phòng một đoạn ghi rõ cách tính, chép gửi Zalo cho người thuê.</t>
   </si>
   <si>
@@ -113,6 +116,9 @@
   </si>
   <si>
     <t xml:space="preserve">KIỂM TRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cách chia điện tháng này</t>
   </si>
   <si>
     <t xml:space="preserve">Phòng</t>
@@ -315,7 +321,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -340,17 +346,17 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <protection locked="false" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -368,6 +374,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="false" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -376,13 +386,9 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+      <protection locked="false" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
@@ -398,6 +404,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -668,7 +678,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="130"/>
@@ -736,26 +746,26 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="A15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="A18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -765,12 +775,12 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
+      <c r="A21" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
@@ -778,15 +788,15 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2"/>
+      <c r="A24" s="4" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -798,6 +808,11 @@
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -814,7 +829,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:G41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -837,20 +852,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="7" t="n">
         <v>1980000</v>
@@ -858,7 +873,7 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>700</v>
@@ -866,16 +881,16 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="9" t="n">
-        <f aca="false">IF(B5&gt;0,B4/B5,0)</f>
+        <f aca="false">IF(N(B5)&gt;0,N(B4)/N(B5),0)</f>
         <v>2828.57142857143</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" s="10" t="n">
         <f aca="false">SUM(E12:E41)</f>
@@ -884,7 +899,7 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">SUM(F12:F41)</f>
@@ -893,42 +908,51 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="12" t="str">
-        <f aca="false">IF(B4&lt;=0,"Nhập số tiền và kWh trên hóa đơn điện lực",IF(SUMPRODUCT(ISTEXT(C12:D41)*(C12:D41&lt;&gt;""))&gt;0,"LỖI: có ô chỉ số điện không phải số (gõ chữ hoặc dấu chấm) – chỉ gõ số",IF(SUMPRODUCT((C12:C41&lt;&gt;"")*(D12:D41&lt;&gt;"")*(D12:D41&lt;C12:C41))&gt;0,"LỖI: có phòng chỉ số điện mới nhỏ hơn chỉ số cũ – kiểm tra lại",IF(B8&gt;B4,"VƯỢT HÓA ĐƠN: đang thu "&amp;TEXT(B8-B4,"#,##0")&amp;" đ nhiều hơn hóa đơn – không được thu",IF(AND(NOT('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng"),B7&gt;B5),"VƯỢT: tổng kWh các phòng lớn hơn kWh trên hóa đơn – kiểm tra chỉ số hoặc công tơ","ĐÚNG: tổng tiền điện thu "&amp;TEXT(B8,"#,##0")&amp;" đ ≤ hóa đơn "&amp;TEXT(B4,"#,##0")&amp;" đ")))))</f>
+        <f aca="false">IF(OR(ISTEXT(B4),ISTEXT(B5)),"LỖI: ô hóa đơn phải là số (không gõ dấu chấm) – vd 1980000",IF(N(B4)&lt;=0,"Nhập số tiền và kWh trên hóa đơn điện lực",IF(SUMPRODUCT((A12:A41&lt;&gt;"")*(D12:D41&lt;&gt;"")*(C12:C41=""))&gt;0,"LỖI: có phòng thiếu chỉ số điện cũ (tháng trước chưa nhập?) – nhập chỉ số cũ",IF(SUMPRODUCT((A12:A41&lt;&gt;"")*(D12:D41=""))&gt;0,"LỖI: có phòng đang thuê chưa nhập chỉ số điện mới",IF(SUMPRODUCT(ISTEXT(C12:D41)*(C12:D41&lt;&gt;""))&gt;0,"LỖI: có ô chỉ số điện không phải số (gõ chữ hoặc dấu chấm) – chỉ gõ số",IF(SUMPRODUCT((C12:C41&lt;&gt;"")*(D12:D41&lt;&gt;"")*(D12:D41&lt;C12:C41))&gt;0,"LỖI: có phòng chỉ số điện mới nhỏ hơn chỉ số cũ – kiểm tra lại",IF(B8&gt;B4,"VƯỢT HÓA ĐƠN: đang thu "&amp;TEXT(B8-B4,"#,##0")&amp;" đ nhiều hơn hóa đơn – không được thu",IF(B7&gt;B5,"VƯỢT: tổng kWh các phòng lớn hơn kWh trên hóa đơn – kiểm tra chỉ số hoặc công tơ","ĐÚNG: tổng tiền điện thu "&amp;TEXT(B8,"#,##0")&amp;" đ ≤ hóa đơn "&amp;TEXT(B4,"#,##0")&amp;" đ"))))))))</f>
         <v>ĐÚNG: tổng tiền điện thu 1,852,600 đ ≤ hóa đơn 1,980,000 đ</v>
       </c>
     </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13" t="str">
+        <f aca="false">'Cài đặt'!B4</f>
+        <v>Giá bình quân hóa đơn (khuyên dùng)</v>
+      </c>
+    </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C11" s="13" t="s">
+      <c r="A11" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="B11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="C11" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="D11" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="E11" s="14" t="s">
         <v>36</v>
       </c>
+      <c r="F11" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>38</v>
+      <c r="A12" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>40</v>
       </c>
       <c r="C12" s="16" t="n">
         <v>1200</v>
@@ -941,22 +965,22 @@
         <v>220</v>
       </c>
       <c r="F12" s="18" t="n">
-        <f aca="false">IF(E12=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E12/$B$7,-2),0),ROUNDDOWN(E12*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E12=0,NOT(OR(A12&lt;&gt;"",B12&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E12/$B$7,-2),0),ROUNDDOWN(E12*$B$6,-2)))</f>
         <v>622200</v>
       </c>
       <c r="G12" s="19" t="str">
-        <f aca="false">IF(OR(A12="",$B$4&lt;=0),"","Phòng "&amp;A12&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C12,"#,##0")&amp;" → "&amp;TEXT(D12,"#,##0")&amp;" = "&amp;E12&amp;" kWh → "&amp;TEXT(F12,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E12&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A12="",$B$4&lt;=0),"","Phòng "&amp;A12&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C12,"#,##0")&amp;" → "&amp;TEXT(D12,"#,##0")&amp;" = "&amp;E12&amp;" kWh → "&amp;TEXT(F12,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E12&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v>Phòng P101 – tháng 10/2026
 Điện: 1,200 → 1,420 = 220 kWh → 622,200 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>40</v>
+      <c r="A13" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="C13" s="16" t="n">
         <v>850</v>
@@ -969,22 +993,22 @@
         <v>140</v>
       </c>
       <c r="F13" s="18" t="n">
-        <f aca="false">IF(E13=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E13/$B$7,-2),0),ROUNDDOWN(E13*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E13=0,NOT(OR(A13&lt;&gt;"",B13&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E13/$B$7,-2),0),ROUNDDOWN(E13*$B$6,-2)))</f>
         <v>396000</v>
       </c>
       <c r="G13" s="19" t="str">
-        <f aca="false">IF(OR(A13="",$B$4&lt;=0),"","Phòng "&amp;A13&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C13,"#,##0")&amp;" → "&amp;TEXT(D13,"#,##0")&amp;" = "&amp;E13&amp;" kWh → "&amp;TEXT(F13,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E13&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A13="",$B$4&lt;=0),"","Phòng "&amp;A13&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C13,"#,##0")&amp;" → "&amp;TEXT(D13,"#,##0")&amp;" = "&amp;E13&amp;" kWh → "&amp;TEXT(F13,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E13&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v>Phòng P102 – tháng 10/2026
 Điện: 850 → 990 = 140 kWh → 396,000 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>42</v>
+      <c r="A14" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>44</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>3010</v>
@@ -997,19 +1021,19 @@
         <v>295</v>
       </c>
       <c r="F14" s="18" t="n">
-        <f aca="false">IF(E14=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E14/$B$7,-2),0),ROUNDDOWN(E14*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E14=0,NOT(OR(A14&lt;&gt;"",B14&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E14/$B$7,-2),0),ROUNDDOWN(E14*$B$6,-2)))</f>
         <v>834400</v>
       </c>
       <c r="G14" s="19" t="str">
-        <f aca="false">IF(OR(A14="",$B$4&lt;=0),"","Phòng "&amp;A14&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C14,"#,##0")&amp;" → "&amp;TEXT(D14,"#,##0")&amp;" = "&amp;E14&amp;" kWh → "&amp;TEXT(F14,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E14&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A14="",$B$4&lt;=0),"","Phòng "&amp;A14&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C14,"#,##0")&amp;" → "&amp;TEXT(D14,"#,##0")&amp;" = "&amp;E14&amp;" kWh → "&amp;TEXT(F14,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E14&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v>Phòng P103 – tháng 10/2026
 Điện: 3,010 → 3,305 = 295 kWh → 834,400 đ
 (Hóa đơn điện lực tháng: 1,980,000 đ / 700 kWh = 2,829 đ/kWh bình quân; làm tròn xuống 100 đ)</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
+      <c r="A15" s="13"/>
+      <c r="B15" s="13"/>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="17" t="n">
@@ -1017,17 +1041,17 @@
         <v>0</v>
       </c>
       <c r="F15" s="18" t="n">
-        <f aca="false">IF(E15=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E15/$B$7,-2),0),ROUNDDOWN(E15*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E15=0,NOT(OR(A15&lt;&gt;"",B15&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E15/$B$7,-2),0),ROUNDDOWN(E15*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G15" s="19" t="str">
-        <f aca="false">IF(OR(A15="",$B$4&lt;=0),"","Phòng "&amp;A15&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C15,"#,##0")&amp;" → "&amp;TEXT(D15,"#,##0")&amp;" = "&amp;E15&amp;" kWh → "&amp;TEXT(F15,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E15&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A15="",$B$4&lt;=0),"","Phòng "&amp;A15&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C15,"#,##0")&amp;" → "&amp;TEXT(D15,"#,##0")&amp;" = "&amp;E15&amp;" kWh → "&amp;TEXT(F15,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E15&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
+      <c r="A16" s="13"/>
+      <c r="B16" s="13"/>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="17" t="n">
@@ -1035,17 +1059,17 @@
         <v>0</v>
       </c>
       <c r="F16" s="18" t="n">
-        <f aca="false">IF(E16=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E16/$B$7,-2),0),ROUNDDOWN(E16*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E16=0,NOT(OR(A16&lt;&gt;"",B16&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E16/$B$7,-2),0),ROUNDDOWN(E16*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G16" s="19" t="str">
-        <f aca="false">IF(OR(A16="",$B$4&lt;=0),"","Phòng "&amp;A16&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C16,"#,##0")&amp;" → "&amp;TEXT(D16,"#,##0")&amp;" = "&amp;E16&amp;" kWh → "&amp;TEXT(F16,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E16&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A16="",$B$4&lt;=0),"","Phòng "&amp;A16&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C16,"#,##0")&amp;" → "&amp;TEXT(D16,"#,##0")&amp;" = "&amp;E16&amp;" kWh → "&amp;TEXT(F16,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E16&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
+      <c r="A17" s="13"/>
+      <c r="B17" s="13"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="17" t="n">
@@ -1053,17 +1077,17 @@
         <v>0</v>
       </c>
       <c r="F17" s="18" t="n">
-        <f aca="false">IF(E17=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E17/$B$7,-2),0),ROUNDDOWN(E17*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E17=0,NOT(OR(A17&lt;&gt;"",B17&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E17/$B$7,-2),0),ROUNDDOWN(E17*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G17" s="19" t="str">
-        <f aca="false">IF(OR(A17="",$B$4&lt;=0),"","Phòng "&amp;A17&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C17,"#,##0")&amp;" → "&amp;TEXT(D17,"#,##0")&amp;" = "&amp;E17&amp;" kWh → "&amp;TEXT(F17,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E17&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A17="",$B$4&lt;=0),"","Phòng "&amp;A17&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C17,"#,##0")&amp;" → "&amp;TEXT(D17,"#,##0")&amp;" = "&amp;E17&amp;" kWh → "&amp;TEXT(F17,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E17&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
+      <c r="A18" s="13"/>
+      <c r="B18" s="13"/>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
       <c r="E18" s="17" t="n">
@@ -1071,17 +1095,17 @@
         <v>0</v>
       </c>
       <c r="F18" s="18" t="n">
-        <f aca="false">IF(E18=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E18/$B$7,-2),0),ROUNDDOWN(E18*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E18=0,NOT(OR(A18&lt;&gt;"",B18&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E18/$B$7,-2),0),ROUNDDOWN(E18*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G18" s="19" t="str">
-        <f aca="false">IF(OR(A18="",$B$4&lt;=0),"","Phòng "&amp;A18&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C18,"#,##0")&amp;" → "&amp;TEXT(D18,"#,##0")&amp;" = "&amp;E18&amp;" kWh → "&amp;TEXT(F18,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E18&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A18="",$B$4&lt;=0),"","Phòng "&amp;A18&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C18,"#,##0")&amp;" → "&amp;TEXT(D18,"#,##0")&amp;" = "&amp;E18&amp;" kWh → "&amp;TEXT(F18,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E18&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
+      <c r="A19" s="13"/>
+      <c r="B19" s="13"/>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
       <c r="E19" s="17" t="n">
@@ -1089,17 +1113,17 @@
         <v>0</v>
       </c>
       <c r="F19" s="18" t="n">
-        <f aca="false">IF(E19=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E19/$B$7,-2),0),ROUNDDOWN(E19*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E19=0,NOT(OR(A19&lt;&gt;"",B19&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E19/$B$7,-2),0),ROUNDDOWN(E19*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G19" s="19" t="str">
-        <f aca="false">IF(OR(A19="",$B$4&lt;=0),"","Phòng "&amp;A19&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C19,"#,##0")&amp;" → "&amp;TEXT(D19,"#,##0")&amp;" = "&amp;E19&amp;" kWh → "&amp;TEXT(F19,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E19&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A19="",$B$4&lt;=0),"","Phòng "&amp;A19&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C19,"#,##0")&amp;" → "&amp;TEXT(D19,"#,##0")&amp;" = "&amp;E19&amp;" kWh → "&amp;TEXT(F19,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E19&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="13"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
       <c r="E20" s="17" t="n">
@@ -1107,17 +1131,17 @@
         <v>0</v>
       </c>
       <c r="F20" s="18" t="n">
-        <f aca="false">IF(E20=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E20/$B$7,-2),0),ROUNDDOWN(E20*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E20=0,NOT(OR(A20&lt;&gt;"",B20&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E20/$B$7,-2),0),ROUNDDOWN(E20*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G20" s="19" t="str">
-        <f aca="false">IF(OR(A20="",$B$4&lt;=0),"","Phòng "&amp;A20&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C20,"#,##0")&amp;" → "&amp;TEXT(D20,"#,##0")&amp;" = "&amp;E20&amp;" kWh → "&amp;TEXT(F20,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E20&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A20="",$B$4&lt;=0),"","Phòng "&amp;A20&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C20,"#,##0")&amp;" → "&amp;TEXT(D20,"#,##0")&amp;" = "&amp;E20&amp;" kWh → "&amp;TEXT(F20,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E20&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="17" t="n">
@@ -1125,17 +1149,17 @@
         <v>0</v>
       </c>
       <c r="F21" s="18" t="n">
-        <f aca="false">IF(E21=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E21/$B$7,-2),0),ROUNDDOWN(E21*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E21=0,NOT(OR(A21&lt;&gt;"",B21&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E21/$B$7,-2),0),ROUNDDOWN(E21*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G21" s="19" t="str">
-        <f aca="false">IF(OR(A21="",$B$4&lt;=0),"","Phòng "&amp;A21&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C21,"#,##0")&amp;" → "&amp;TEXT(D21,"#,##0")&amp;" = "&amp;E21&amp;" kWh → "&amp;TEXT(F21,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E21&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A21="",$B$4&lt;=0),"","Phòng "&amp;A21&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C21,"#,##0")&amp;" → "&amp;TEXT(D21,"#,##0")&amp;" = "&amp;E21&amp;" kWh → "&amp;TEXT(F21,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E21&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="13"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="17" t="n">
@@ -1143,17 +1167,17 @@
         <v>0</v>
       </c>
       <c r="F22" s="18" t="n">
-        <f aca="false">IF(E22=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E22/$B$7,-2),0),ROUNDDOWN(E22*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E22=0,NOT(OR(A22&lt;&gt;"",B22&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E22/$B$7,-2),0),ROUNDDOWN(E22*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G22" s="19" t="str">
-        <f aca="false">IF(OR(A22="",$B$4&lt;=0),"","Phòng "&amp;A22&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C22,"#,##0")&amp;" → "&amp;TEXT(D22,"#,##0")&amp;" = "&amp;E22&amp;" kWh → "&amp;TEXT(F22,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E22&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A22="",$B$4&lt;=0),"","Phòng "&amp;A22&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C22,"#,##0")&amp;" → "&amp;TEXT(D22,"#,##0")&amp;" = "&amp;E22&amp;" kWh → "&amp;TEXT(F22,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E22&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15"/>
-      <c r="B23" s="15"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="13"/>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
       <c r="E23" s="17" t="n">
@@ -1161,17 +1185,17 @@
         <v>0</v>
       </c>
       <c r="F23" s="18" t="n">
-        <f aca="false">IF(E23=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E23/$B$7,-2),0),ROUNDDOWN(E23*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E23=0,NOT(OR(A23&lt;&gt;"",B23&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E23/$B$7,-2),0),ROUNDDOWN(E23*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G23" s="19" t="str">
-        <f aca="false">IF(OR(A23="",$B$4&lt;=0),"","Phòng "&amp;A23&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C23,"#,##0")&amp;" → "&amp;TEXT(D23,"#,##0")&amp;" = "&amp;E23&amp;" kWh → "&amp;TEXT(F23,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E23&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A23="",$B$4&lt;=0),"","Phòng "&amp;A23&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C23,"#,##0")&amp;" → "&amp;TEXT(D23,"#,##0")&amp;" = "&amp;E23&amp;" kWh → "&amp;TEXT(F23,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E23&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="13"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="17" t="n">
@@ -1179,17 +1203,17 @@
         <v>0</v>
       </c>
       <c r="F24" s="18" t="n">
-        <f aca="false">IF(E24=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E24/$B$7,-2),0),ROUNDDOWN(E24*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E24=0,NOT(OR(A24&lt;&gt;"",B24&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E24/$B$7,-2),0),ROUNDDOWN(E24*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G24" s="19" t="str">
-        <f aca="false">IF(OR(A24="",$B$4&lt;=0),"","Phòng "&amp;A24&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C24,"#,##0")&amp;" → "&amp;TEXT(D24,"#,##0")&amp;" = "&amp;E24&amp;" kWh → "&amp;TEXT(F24,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E24&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A24="",$B$4&lt;=0),"","Phòng "&amp;A24&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C24,"#,##0")&amp;" → "&amp;TEXT(D24,"#,##0")&amp;" = "&amp;E24&amp;" kWh → "&amp;TEXT(F24,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E24&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="13"/>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="17" t="n">
@@ -1197,17 +1221,17 @@
         <v>0</v>
       </c>
       <c r="F25" s="18" t="n">
-        <f aca="false">IF(E25=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E25/$B$7,-2),0),ROUNDDOWN(E25*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E25=0,NOT(OR(A25&lt;&gt;"",B25&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E25/$B$7,-2),0),ROUNDDOWN(E25*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G25" s="19" t="str">
-        <f aca="false">IF(OR(A25="",$B$4&lt;=0),"","Phòng "&amp;A25&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C25,"#,##0")&amp;" → "&amp;TEXT(D25,"#,##0")&amp;" = "&amp;E25&amp;" kWh → "&amp;TEXT(F25,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E25&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A25="",$B$4&lt;=0),"","Phòng "&amp;A25&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C25,"#,##0")&amp;" → "&amp;TEXT(D25,"#,##0")&amp;" = "&amp;E25&amp;" kWh → "&amp;TEXT(F25,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E25&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="13"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="17" t="n">
@@ -1215,17 +1239,17 @@
         <v>0</v>
       </c>
       <c r="F26" s="18" t="n">
-        <f aca="false">IF(E26=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E26/$B$7,-2),0),ROUNDDOWN(E26*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E26=0,NOT(OR(A26&lt;&gt;"",B26&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E26/$B$7,-2),0),ROUNDDOWN(E26*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G26" s="19" t="str">
-        <f aca="false">IF(OR(A26="",$B$4&lt;=0),"","Phòng "&amp;A26&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C26,"#,##0")&amp;" → "&amp;TEXT(D26,"#,##0")&amp;" = "&amp;E26&amp;" kWh → "&amp;TEXT(F26,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E26&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A26="",$B$4&lt;=0),"","Phòng "&amp;A26&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C26,"#,##0")&amp;" → "&amp;TEXT(D26,"#,##0")&amp;" = "&amp;E26&amp;" kWh → "&amp;TEXT(F26,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E26&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="13"/>
       <c r="C27" s="16"/>
       <c r="D27" s="16"/>
       <c r="E27" s="17" t="n">
@@ -1233,17 +1257,17 @@
         <v>0</v>
       </c>
       <c r="F27" s="18" t="n">
-        <f aca="false">IF(E27=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E27/$B$7,-2),0),ROUNDDOWN(E27*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E27=0,NOT(OR(A27&lt;&gt;"",B27&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E27/$B$7,-2),0),ROUNDDOWN(E27*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G27" s="19" t="str">
-        <f aca="false">IF(OR(A27="",$B$4&lt;=0),"","Phòng "&amp;A27&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C27,"#,##0")&amp;" → "&amp;TEXT(D27,"#,##0")&amp;" = "&amp;E27&amp;" kWh → "&amp;TEXT(F27,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E27&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A27="",$B$4&lt;=0),"","Phòng "&amp;A27&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C27,"#,##0")&amp;" → "&amp;TEXT(D27,"#,##0")&amp;" = "&amp;E27&amp;" kWh → "&amp;TEXT(F27,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E27&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="13"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
       <c r="E28" s="17" t="n">
@@ -1251,17 +1275,17 @@
         <v>0</v>
       </c>
       <c r="F28" s="18" t="n">
-        <f aca="false">IF(E28=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E28/$B$7,-2),0),ROUNDDOWN(E28*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E28=0,NOT(OR(A28&lt;&gt;"",B28&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E28/$B$7,-2),0),ROUNDDOWN(E28*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G28" s="19" t="str">
-        <f aca="false">IF(OR(A28="",$B$4&lt;=0),"","Phòng "&amp;A28&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C28,"#,##0")&amp;" → "&amp;TEXT(D28,"#,##0")&amp;" = "&amp;E28&amp;" kWh → "&amp;TEXT(F28,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E28&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A28="",$B$4&lt;=0),"","Phòng "&amp;A28&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C28,"#,##0")&amp;" → "&amp;TEXT(D28,"#,##0")&amp;" = "&amp;E28&amp;" kWh → "&amp;TEXT(F28,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E28&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
       <c r="E29" s="17" t="n">
@@ -1269,17 +1293,17 @@
         <v>0</v>
       </c>
       <c r="F29" s="18" t="n">
-        <f aca="false">IF(E29=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E29/$B$7,-2),0),ROUNDDOWN(E29*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E29=0,NOT(OR(A29&lt;&gt;"",B29&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E29/$B$7,-2),0),ROUNDDOWN(E29*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G29" s="19" t="str">
-        <f aca="false">IF(OR(A29="",$B$4&lt;=0),"","Phòng "&amp;A29&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C29,"#,##0")&amp;" → "&amp;TEXT(D29,"#,##0")&amp;" = "&amp;E29&amp;" kWh → "&amp;TEXT(F29,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E29&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A29="",$B$4&lt;=0),"","Phòng "&amp;A29&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C29,"#,##0")&amp;" → "&amp;TEXT(D29,"#,##0")&amp;" = "&amp;E29&amp;" kWh → "&amp;TEXT(F29,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E29&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15"/>
-      <c r="B30" s="15"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
       <c r="E30" s="17" t="n">
@@ -1287,17 +1311,17 @@
         <v>0</v>
       </c>
       <c r="F30" s="18" t="n">
-        <f aca="false">IF(E30=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E30/$B$7,-2),0),ROUNDDOWN(E30*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E30=0,NOT(OR(A30&lt;&gt;"",B30&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E30/$B$7,-2),0),ROUNDDOWN(E30*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G30" s="19" t="str">
-        <f aca="false">IF(OR(A30="",$B$4&lt;=0),"","Phòng "&amp;A30&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C30,"#,##0")&amp;" → "&amp;TEXT(D30,"#,##0")&amp;" = "&amp;E30&amp;" kWh → "&amp;TEXT(F30,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E30&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A30="",$B$4&lt;=0),"","Phòng "&amp;A30&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C30,"#,##0")&amp;" → "&amp;TEXT(D30,"#,##0")&amp;" = "&amp;E30&amp;" kWh → "&amp;TEXT(F30,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E30&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15"/>
-      <c r="B31" s="15"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
       <c r="C31" s="16"/>
       <c r="D31" s="16"/>
       <c r="E31" s="17" t="n">
@@ -1305,17 +1329,17 @@
         <v>0</v>
       </c>
       <c r="F31" s="18" t="n">
-        <f aca="false">IF(E31=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E31/$B$7,-2),0),ROUNDDOWN(E31*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E31=0,NOT(OR(A31&lt;&gt;"",B31&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E31/$B$7,-2),0),ROUNDDOWN(E31*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G31" s="19" t="str">
-        <f aca="false">IF(OR(A31="",$B$4&lt;=0),"","Phòng "&amp;A31&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C31,"#,##0")&amp;" → "&amp;TEXT(D31,"#,##0")&amp;" = "&amp;E31&amp;" kWh → "&amp;TEXT(F31,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E31&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A31="",$B$4&lt;=0),"","Phòng "&amp;A31&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C31,"#,##0")&amp;" → "&amp;TEXT(D31,"#,##0")&amp;" = "&amp;E31&amp;" kWh → "&amp;TEXT(F31,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E31&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15"/>
-      <c r="B32" s="15"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="17" t="n">
@@ -1323,17 +1347,17 @@
         <v>0</v>
       </c>
       <c r="F32" s="18" t="n">
-        <f aca="false">IF(E32=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E32/$B$7,-2),0),ROUNDDOWN(E32*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E32=0,NOT(OR(A32&lt;&gt;"",B32&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E32/$B$7,-2),0),ROUNDDOWN(E32*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G32" s="19" t="str">
-        <f aca="false">IF(OR(A32="",$B$4&lt;=0),"","Phòng "&amp;A32&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C32,"#,##0")&amp;" → "&amp;TEXT(D32,"#,##0")&amp;" = "&amp;E32&amp;" kWh → "&amp;TEXT(F32,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E32&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A32="",$B$4&lt;=0),"","Phòng "&amp;A32&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C32,"#,##0")&amp;" → "&amp;TEXT(D32,"#,##0")&amp;" = "&amp;E32&amp;" kWh → "&amp;TEXT(F32,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E32&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15"/>
-      <c r="B33" s="15"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="13"/>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
       <c r="E33" s="17" t="n">
@@ -1341,17 +1365,17 @@
         <v>0</v>
       </c>
       <c r="F33" s="18" t="n">
-        <f aca="false">IF(E33=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E33/$B$7,-2),0),ROUNDDOWN(E33*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E33=0,NOT(OR(A33&lt;&gt;"",B33&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E33/$B$7,-2),0),ROUNDDOWN(E33*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G33" s="19" t="str">
-        <f aca="false">IF(OR(A33="",$B$4&lt;=0),"","Phòng "&amp;A33&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C33,"#,##0")&amp;" → "&amp;TEXT(D33,"#,##0")&amp;" = "&amp;E33&amp;" kWh → "&amp;TEXT(F33,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E33&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A33="",$B$4&lt;=0),"","Phòng "&amp;A33&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C33,"#,##0")&amp;" → "&amp;TEXT(D33,"#,##0")&amp;" = "&amp;E33&amp;" kWh → "&amp;TEXT(F33,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E33&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15"/>
-      <c r="B34" s="15"/>
+      <c r="A34" s="13"/>
+      <c r="B34" s="13"/>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
       <c r="E34" s="17" t="n">
@@ -1359,17 +1383,17 @@
         <v>0</v>
       </c>
       <c r="F34" s="18" t="n">
-        <f aca="false">IF(E34=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E34/$B$7,-2),0),ROUNDDOWN(E34*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E34=0,NOT(OR(A34&lt;&gt;"",B34&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E34/$B$7,-2),0),ROUNDDOWN(E34*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G34" s="19" t="str">
-        <f aca="false">IF(OR(A34="",$B$4&lt;=0),"","Phòng "&amp;A34&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C34,"#,##0")&amp;" → "&amp;TEXT(D34,"#,##0")&amp;" = "&amp;E34&amp;" kWh → "&amp;TEXT(F34,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E34&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A34="",$B$4&lt;=0),"","Phòng "&amp;A34&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C34,"#,##0")&amp;" → "&amp;TEXT(D34,"#,##0")&amp;" = "&amp;E34&amp;" kWh → "&amp;TEXT(F34,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E34&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15"/>
-      <c r="B35" s="15"/>
+      <c r="A35" s="13"/>
+      <c r="B35" s="13"/>
       <c r="C35" s="16"/>
       <c r="D35" s="16"/>
       <c r="E35" s="17" t="n">
@@ -1377,17 +1401,17 @@
         <v>0</v>
       </c>
       <c r="F35" s="18" t="n">
-        <f aca="false">IF(E35=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E35/$B$7,-2),0),ROUNDDOWN(E35*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E35=0,NOT(OR(A35&lt;&gt;"",B35&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E35/$B$7,-2),0),ROUNDDOWN(E35*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G35" s="19" t="str">
-        <f aca="false">IF(OR(A35="",$B$4&lt;=0),"","Phòng "&amp;A35&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C35,"#,##0")&amp;" → "&amp;TEXT(D35,"#,##0")&amp;" = "&amp;E35&amp;" kWh → "&amp;TEXT(F35,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E35&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A35="",$B$4&lt;=0),"","Phòng "&amp;A35&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C35,"#,##0")&amp;" → "&amp;TEXT(D35,"#,##0")&amp;" = "&amp;E35&amp;" kWh → "&amp;TEXT(F35,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E35&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15"/>
-      <c r="B36" s="15"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="13"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="17" t="n">
@@ -1395,17 +1419,17 @@
         <v>0</v>
       </c>
       <c r="F36" s="18" t="n">
-        <f aca="false">IF(E36=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E36/$B$7,-2),0),ROUNDDOWN(E36*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E36=0,NOT(OR(A36&lt;&gt;"",B36&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E36/$B$7,-2),0),ROUNDDOWN(E36*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G36" s="19" t="str">
-        <f aca="false">IF(OR(A36="",$B$4&lt;=0),"","Phòng "&amp;A36&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C36,"#,##0")&amp;" → "&amp;TEXT(D36,"#,##0")&amp;" = "&amp;E36&amp;" kWh → "&amp;TEXT(F36,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E36&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A36="",$B$4&lt;=0),"","Phòng "&amp;A36&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C36,"#,##0")&amp;" → "&amp;TEXT(D36,"#,##0")&amp;" = "&amp;E36&amp;" kWh → "&amp;TEXT(F36,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E36&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15"/>
-      <c r="B37" s="15"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="13"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="E37" s="17" t="n">
@@ -1413,17 +1437,17 @@
         <v>0</v>
       </c>
       <c r="F37" s="18" t="n">
-        <f aca="false">IF(E37=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E37/$B$7,-2),0),ROUNDDOWN(E37*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E37=0,NOT(OR(A37&lt;&gt;"",B37&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E37/$B$7,-2),0),ROUNDDOWN(E37*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G37" s="19" t="str">
-        <f aca="false">IF(OR(A37="",$B$4&lt;=0),"","Phòng "&amp;A37&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C37,"#,##0")&amp;" → "&amp;TEXT(D37,"#,##0")&amp;" = "&amp;E37&amp;" kWh → "&amp;TEXT(F37,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E37&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A37="",$B$4&lt;=0),"","Phòng "&amp;A37&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C37,"#,##0")&amp;" → "&amp;TEXT(D37,"#,##0")&amp;" = "&amp;E37&amp;" kWh → "&amp;TEXT(F37,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E37&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="13"/>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="17" t="n">
@@ -1431,17 +1455,17 @@
         <v>0</v>
       </c>
       <c r="F38" s="18" t="n">
-        <f aca="false">IF(E38=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E38/$B$7,-2),0),ROUNDDOWN(E38*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E38=0,NOT(OR(A38&lt;&gt;"",B38&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E38/$B$7,-2),0),ROUNDDOWN(E38*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G38" s="19" t="str">
-        <f aca="false">IF(OR(A38="",$B$4&lt;=0),"","Phòng "&amp;A38&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C38,"#,##0")&amp;" → "&amp;TEXT(D38,"#,##0")&amp;" = "&amp;E38&amp;" kWh → "&amp;TEXT(F38,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E38&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A38="",$B$4&lt;=0),"","Phòng "&amp;A38&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C38,"#,##0")&amp;" → "&amp;TEXT(D38,"#,##0")&amp;" = "&amp;E38&amp;" kWh → "&amp;TEXT(F38,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E38&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15"/>
-      <c r="B39" s="15"/>
+      <c r="A39" s="13"/>
+      <c r="B39" s="13"/>
       <c r="C39" s="16"/>
       <c r="D39" s="16"/>
       <c r="E39" s="17" t="n">
@@ -1449,17 +1473,17 @@
         <v>0</v>
       </c>
       <c r="F39" s="18" t="n">
-        <f aca="false">IF(E39=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E39/$B$7,-2),0),ROUNDDOWN(E39*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E39=0,NOT(OR(A39&lt;&gt;"",B39&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E39/$B$7,-2),0),ROUNDDOWN(E39*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G39" s="19" t="str">
-        <f aca="false">IF(OR(A39="",$B$4&lt;=0),"","Phòng "&amp;A39&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C39,"#,##0")&amp;" → "&amp;TEXT(D39,"#,##0")&amp;" = "&amp;E39&amp;" kWh → "&amp;TEXT(F39,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E39&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A39="",$B$4&lt;=0),"","Phòng "&amp;A39&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C39,"#,##0")&amp;" → "&amp;TEXT(D39,"#,##0")&amp;" = "&amp;E39&amp;" kWh → "&amp;TEXT(F39,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E39&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15"/>
-      <c r="B40" s="15"/>
+      <c r="A40" s="13"/>
+      <c r="B40" s="13"/>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="17" t="n">
@@ -1467,17 +1491,17 @@
         <v>0</v>
       </c>
       <c r="F40" s="18" t="n">
-        <f aca="false">IF(E40=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E40/$B$7,-2),0),ROUNDDOWN(E40*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E40=0,NOT(OR(A40&lt;&gt;"",B40&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E40/$B$7,-2),0),ROUNDDOWN(E40*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G40" s="19" t="str">
-        <f aca="false">IF(OR(A40="",$B$4&lt;=0),"","Phòng "&amp;A40&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C40,"#,##0")&amp;" → "&amp;TEXT(D40,"#,##0")&amp;" = "&amp;E40&amp;" kWh → "&amp;TEXT(F40,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E40&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A40="",$B$4&lt;=0),"","Phòng "&amp;A40&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C40,"#,##0")&amp;" → "&amp;TEXT(D40,"#,##0")&amp;" = "&amp;E40&amp;" kWh → "&amp;TEXT(F40,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E40&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15"/>
-      <c r="B41" s="15"/>
+      <c r="A41" s="13"/>
+      <c r="B41" s="13"/>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="17" t="n">
@@ -1485,15 +1509,16 @@
         <v>0</v>
       </c>
       <c r="F41" s="18" t="n">
-        <f aca="false">IF(E41=0,0,IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN($B$4*E41/$B$7,-2),0),ROUNDDOWN(E41*$B$6,-2)))</f>
+        <f aca="false">IF(OR(E41=0,NOT(OR(A41&lt;&gt;"",B41&lt;&gt;""))),0,IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng",IF($B$7&gt;0,ROUNDDOWN(N($B$4)*E41/$B$7,-2),0),ROUNDDOWN(E41*$B$6,-2)))</f>
         <v>0</v>
       </c>
       <c r="G41" s="19" t="str">
-        <f aca="false">IF(OR(A41="",$B$4&lt;=0),"","Phòng "&amp;A41&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C41,"#,##0")&amp;" → "&amp;TEXT(D41,"#,##0")&amp;" = "&amp;E41&amp;" kWh → "&amp;TEXT(F41,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF('Cài đặt'!$B$4="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E41&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
+        <f aca="false">IF(OR(A41="",$B$4&lt;=0),"","Phòng "&amp;A41&amp;" – tháng "&amp;$B$3&amp;CHAR(10)&amp;"Điện: "&amp;TEXT(C41,"#,##0")&amp;" → "&amp;TEXT(D41,"#,##0")&amp;" = "&amp;E41&amp;" kWh → "&amp;TEXT(F41,"#,##0")&amp;" đ"&amp;CHAR(10)&amp;IF($B$10="Chia hết hóa đơn theo tỷ lệ dùng","(Chia hóa đơn điện lực "&amp;TEXT($B$4,"#,##0")&amp;" đ theo tỷ lệ: phòng dùng "&amp;E41&amp;" / tổng các phòng "&amp;TEXT($B$7,"#,##0")&amp;" kWh; làm tròn xuống 100 đ)","(Hóa đơn điện lực tháng: "&amp;TEXT($B$4,"#,##0")&amp;" đ / "&amp;TEXT($B$5,"#,##0")&amp;" kWh = "&amp;TEXT($B$6,"#,##0")&amp;" đ/kWh bình quân; làm tròn xuống 100 đ)"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false"/>
   <conditionalFormatting sqref="B9">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEFT(B9,4)="ĐÚNG"</formula>
@@ -1507,7 +1532,11 @@
       <formula>AND(C12&lt;&gt;"",D12&lt;&gt;"",D12&lt;C12)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B10" type="list">
+      <formula1>"Giá bình quân hóa đơn (khuyên dùng),Chia hết hóa đơn theo tỷ lệ dùng"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
     <dataValidation allowBlank="false" error="Nhập số, không âm" errorStyle="stop" operator="greaterThanOrEqual" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B4:B5 C12:D41" type="decimal">
       <formula1>0</formula1>
       <formula2>0</formula2>
@@ -1515,7 +1544,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1526,7 +1555,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:A32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -1536,12 +1565,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1733,7 +1762,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1755,23 +1784,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>